<commit_message>
add ffa column to dairy test threshold report
</commit_message>
<xml_diff>
--- a/backend/src/static/templates/reports/Dairy_Test_Threshold_Template.xlsx
+++ b/backend/src/static/templates/reports/Dairy_Test_Threshold_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gh\nr-mals\app\server\static\templates\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gh\nr-mals\backend\src\static\templates\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B7213E-3B24-4304-B368-7A7A03999F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6361B21C-0749-480A-AC94-B341ED633889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{11309506-049F-4A42-8D72-2555D662D497}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{11309506-049F-4A42-8D72-2555D662D497}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Threshold Report" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>Client</t>
   </si>
@@ -126,6 +126,15 @@
   </si>
   <si>
     <t>{d.Reg[i].PenaltyIssued}</t>
+  </si>
+  <si>
+    <t>FFA Threshold 1.2</t>
+  </si>
+  <si>
+    <t>{d.Reg[i].FFA_Result}</t>
+  </si>
+  <si>
+    <t>{d.Tot_FFA_Count}</t>
   </si>
 </sst>
 </file>
@@ -532,21 +541,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6B4FD09-964A-4163-B64E-5BD98D9AE9F8}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="37" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="12.42578125" customWidth="1"/>
     <col min="9" max="9" width="11.28515625" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>6</v>
       </c>
@@ -560,7 +570,7 @@
       <c r="G1" s="10"/>
       <c r="H1" s="10"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
         <v>8</v>
       </c>
@@ -576,7 +586,7 @@
       <c r="G2" s="16"/>
       <c r="H2" s="16"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -586,8 +596,9 @@
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
       <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
     </row>
-    <row r="4" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>1</v>
       </c>
@@ -613,10 +624,13 @@
         <v>17</v>
       </c>
       <c r="I4" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -626,8 +640,9 @@
       <c r="G5" s="12"/>
       <c r="H5" s="11"/>
       <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
@@ -652,11 +667,14 @@
       <c r="H6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>13</v>
       </c>
@@ -666,22 +684,22 @@
       </c>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C8" s="7"/>
       <c r="D8" s="9"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C9" s="7"/>
       <c r="D9" s="9"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C10" s="7"/>
       <c r="D10" s="9"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
@@ -699,6 +717,9 @@
       </c>
       <c r="H11" s="13" t="s">
         <v>27</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -711,6 +732,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B8CBF3948AF16E4A9427EB9CB0C3AFDB" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0f00dee740a70860da74dc5110d51704">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bc8b8595-9fa1-49bc-a016-2621e7bde64e" xmlns:ns3="e1c8ebbc-f196-4c28-98e9-1900bd408e79" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2351f42212ae562663f11aa838f8e3a4" ns2:_="" ns3:_="">
     <xsd:import namespace="bc8b8595-9fa1-49bc-a016-2621e7bde64e"/>
@@ -933,12 +960,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -949,6 +970,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{028A420A-B050-4A61-806A-8D9C587E3D76}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="bc8b8595-9fa1-49bc-a016-2621e7bde64e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="e1c8ebbc-f196-4c28-98e9-1900bd408e79"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DAC4DD0-6527-4C33-8A5D-F6D18A2872ED}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -967,23 +1005,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{028A420A-B050-4A61-806A-8D9C587E3D76}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="bc8b8595-9fa1-49bc-a016-2621e7bde64e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="e1c8ebbc-f196-4c28-98e9-1900bd408e79"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F54B38D-A965-4592-A05D-BAAD7EF0EFBC}">
   <ds:schemaRefs>

</xml_diff>